<commit_message>
Update Nikkei225 Ver7 research data
</commit_message>
<xml_diff>
--- a/reports/daily/nikkei225_ranking_ver7_20260918.xlsx
+++ b/reports/daily/nikkei225_ranking_ver7_20260918.xlsx
@@ -860,7 +860,7 @@
         <v>1734</v>
       </c>
       <c r="AV2" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="AW2" t="n">
         <v>0</v>
@@ -1045,7 +1045,7 @@
         <v>1187</v>
       </c>
       <c r="AV3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AW3" t="n">
         <v>0</v>
@@ -1230,7 +1230,7 @@
         <v>1771</v>
       </c>
       <c r="AV4" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="AW4" t="n">
         <v>0</v>
@@ -1415,7 +1415,7 @@
         <v>1554</v>
       </c>
       <c r="AV5" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="AW5" t="n">
         <v>0</v>
@@ -1600,7 +1600,7 @@
         <v>4985</v>
       </c>
       <c r="AV6" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="AW6" t="n">
         <v>0</v>
@@ -1785,7 +1785,7 @@
         <v>533.9</v>
       </c>
       <c r="AV7" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="AW7" t="n">
         <v>0</v>
@@ -1970,7 +1970,7 @@
         <v>1675</v>
       </c>
       <c r="AV8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AW8" t="n">
         <v>0</v>
@@ -2155,7 +2155,7 @@
         <v>2957</v>
       </c>
       <c r="AV9" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AW9" t="n">
         <v>0</v>
@@ -2340,7 +2340,7 @@
         <v>7158</v>
       </c>
       <c r="AV10" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AW10" t="n">
         <v>0</v>
@@ -2525,7 +2525,7 @@
         <v>5618</v>
       </c>
       <c r="AV11" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="AW11" t="n">
         <v>0</v>
@@ -2714,7 +2714,7 @@
         <v>8531</v>
       </c>
       <c r="AV12" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="AW12" t="n">
         <v>0</v>
@@ -2903,7 +2903,7 @@
         <v>1833</v>
       </c>
       <c r="AV13" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AW13" t="n">
         <v>0</v>
@@ -3088,7 +3088,7 @@
         <v>7583</v>
       </c>
       <c r="AV14" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="AW14" t="n">
         <v>0</v>
@@ -3273,7 +3273,7 @@
         <v>2837.5</v>
       </c>
       <c r="AV15" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="AW15" t="n">
         <v>0</v>
@@ -3462,7 +3462,7 @@
         <v>173.2</v>
       </c>
       <c r="AV16" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AW16" t="n">
         <v>0</v>
@@ -3651,7 +3651,7 @@
         <v>3654</v>
       </c>
       <c r="AV17" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="AW17" t="n">
         <v>0</v>
@@ -3836,7 +3836,7 @@
         <v>1983.5</v>
       </c>
       <c r="AV18" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AW18" t="n">
         <v>0</v>
@@ -4021,7 +4021,7 @@
         <v>2309</v>
       </c>
       <c r="AV19" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AW19" t="n">
         <v>0</v>
@@ -4206,7 +4206,7 @@
         <v>7564</v>
       </c>
       <c r="AV20" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="AW20" t="n">
         <v>0</v>
@@ -4391,7 +4391,7 @@
         <v>20960</v>
       </c>
       <c r="AV21" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AW21" t="n">
         <v>0</v>
@@ -4580,7 +4580,7 @@
         <v>4682</v>
       </c>
       <c r="AV22" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AW22" t="n">
         <v>0</v>
@@ -4765,7 +4765,7 @@
         <v>16435</v>
       </c>
       <c r="AV23" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="AW23" t="n">
         <v>0</v>
@@ -4954,7 +4954,7 @@
         <v>6834</v>
       </c>
       <c r="AV24" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AW24" t="n">
         <v>0</v>
@@ -5139,7 +5139,7 @@
         <v>1820</v>
       </c>
       <c r="AV25" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="AW25" t="n">
         <v>0</v>
@@ -5328,7 +5328,7 @@
         <v>6776</v>
       </c>
       <c r="AV26" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="AW26" t="n">
         <v>0</v>
@@ -5683,7 +5683,7 @@
         <v>9</v>
       </c>
       <c r="AW28" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AX28" t="n">
         <v>3.888649734538663</v>
@@ -13464,7 +13464,9 @@
       <c r="I75" t="n">
         <v>4.9</v>
       </c>
-      <c r="J75" t="inlineStr"/>
+      <c r="J75" t="n">
+        <v>45.7</v>
+      </c>
       <c r="K75" t="n">
         <v>1.5</v>
       </c>
@@ -18414,28 +18416,14 @@
       <c r="AR104" t="n">
         <v>103</v>
       </c>
-      <c r="AS104" t="inlineStr">
-        <is>
-          <t>2503_20260917_02</t>
-        </is>
-      </c>
-      <c r="AT104" t="inlineStr">
-        <is>
-          <t>2026-09-17</t>
-        </is>
-      </c>
-      <c r="AU104" t="n">
-        <v>2893.5</v>
-      </c>
-      <c r="AV104" t="n">
+      <c r="AS104" t="inlineStr"/>
+      <c r="AT104" t="inlineStr"/>
+      <c r="AU104" t="inlineStr"/>
+      <c r="AV104" t="inlineStr"/>
+      <c r="AW104" t="n">
         <v>0</v>
       </c>
-      <c r="AW104" t="n">
-        <v>2</v>
-      </c>
-      <c r="AX104" t="n">
-        <v>-1.555209953343706</v>
-      </c>
+      <c r="AX104" t="inlineStr"/>
       <c r="AY104" t="n">
         <v>110</v>
       </c>
@@ -18445,11 +18433,7 @@
       <c r="BA104" t="n">
         <v>0.1999999999999886</v>
       </c>
-      <c r="BB104" t="inlineStr">
-        <is>
-          <t>MATURE</t>
-        </is>
-      </c>
+      <c r="BB104" t="inlineStr"/>
       <c r="BC104" t="inlineStr">
         <is>
           <t>SKIP</t>
@@ -37679,7 +37663,7 @@
         <v>1734</v>
       </c>
       <c r="AV2" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="AW2" t="n">
         <v>0</v>
@@ -37864,7 +37848,7 @@
         <v>1187</v>
       </c>
       <c r="AV3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AW3" t="n">
         <v>0</v>
@@ -38049,7 +38033,7 @@
         <v>1771</v>
       </c>
       <c r="AV4" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="AW4" t="n">
         <v>0</v>
@@ -38234,7 +38218,7 @@
         <v>1554</v>
       </c>
       <c r="AV5" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="AW5" t="n">
         <v>0</v>
@@ -38419,7 +38403,7 @@
         <v>4985</v>
       </c>
       <c r="AV6" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="AW6" t="n">
         <v>0</v>
@@ -38604,7 +38588,7 @@
         <v>533.9</v>
       </c>
       <c r="AV7" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="AW7" t="n">
         <v>0</v>
@@ -38789,7 +38773,7 @@
         <v>1675</v>
       </c>
       <c r="AV8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AW8" t="n">
         <v>0</v>
@@ -38974,7 +38958,7 @@
         <v>2957</v>
       </c>
       <c r="AV9" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AW9" t="n">
         <v>0</v>
@@ -39159,7 +39143,7 @@
         <v>7158</v>
       </c>
       <c r="AV10" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AW10" t="n">
         <v>0</v>
@@ -39344,7 +39328,7 @@
         <v>5618</v>
       </c>
       <c r="AV11" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="AW11" t="n">
         <v>0</v>
@@ -39533,7 +39517,7 @@
         <v>8531</v>
       </c>
       <c r="AV12" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="AW12" t="n">
         <v>0</v>
@@ -39722,7 +39706,7 @@
         <v>1833</v>
       </c>
       <c r="AV13" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AW13" t="n">
         <v>0</v>
@@ -39907,7 +39891,7 @@
         <v>7583</v>
       </c>
       <c r="AV14" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="AW14" t="n">
         <v>0</v>
@@ -40092,7 +40076,7 @@
         <v>2837.5</v>
       </c>
       <c r="AV15" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="AW15" t="n">
         <v>0</v>
@@ -40281,7 +40265,7 @@
         <v>173.2</v>
       </c>
       <c r="AV16" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AW16" t="n">
         <v>0</v>
@@ -40470,7 +40454,7 @@
         <v>3654</v>
       </c>
       <c r="AV17" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="AW17" t="n">
         <v>0</v>
@@ -40655,7 +40639,7 @@
         <v>1983.5</v>
       </c>
       <c r="AV18" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AW18" t="n">
         <v>0</v>
@@ -40840,7 +40824,7 @@
         <v>2309</v>
       </c>
       <c r="AV19" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AW19" t="n">
         <v>0</v>
@@ -41025,7 +41009,7 @@
         <v>7564</v>
       </c>
       <c r="AV20" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="AW20" t="n">
         <v>0</v>
@@ -41210,7 +41194,7 @@
         <v>20960</v>
       </c>
       <c r="AV21" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AW21" t="n">
         <v>0</v>
@@ -41399,7 +41383,7 @@
         <v>4682</v>
       </c>
       <c r="AV22" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AW22" t="n">
         <v>0</v>
@@ -41584,7 +41568,7 @@
         <v>16435</v>
       </c>
       <c r="AV23" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="AW23" t="n">
         <v>0</v>
@@ -41773,7 +41757,7 @@
         <v>6834</v>
       </c>
       <c r="AV24" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AW24" t="n">
         <v>0</v>
@@ -41958,7 +41942,7 @@
         <v>1820</v>
       </c>
       <c r="AV25" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="AW25" t="n">
         <v>0</v>
@@ -42147,7 +42131,7 @@
         <v>6776</v>
       </c>
       <c r="AV26" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="AW26" t="n">
         <v>0</v>
@@ -42627,7 +42611,7 @@
         <v>4682</v>
       </c>
       <c r="AV2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AW2" t="n">
         <v>0</v>
@@ -45831,7 +45815,7 @@
         <v>6834</v>
       </c>
       <c r="AV2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AW2" t="n">
         <v>0</v>
@@ -46020,7 +46004,7 @@
         <v>1833</v>
       </c>
       <c r="AV3" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AW3" t="n">
         <v>0</v>
@@ -46380,7 +46364,7 @@
         <v>173.2</v>
       </c>
       <c r="AV5" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AW5" t="n">
         <v>0</v>
@@ -47082,7 +47066,7 @@
         <v>1734</v>
       </c>
       <c r="AV9" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="AW9" t="n">
         <v>0</v>
@@ -47271,7 +47255,7 @@
         <v>3654</v>
       </c>
       <c r="AV10" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="AW10" t="n">
         <v>0</v>
@@ -47973,7 +47957,7 @@
         <v>8531</v>
       </c>
       <c r="AV14" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="AW14" t="n">
         <v>0</v>
@@ -48502,7 +48486,7 @@
         <v>6776</v>
       </c>
       <c r="AV17" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="AW17" t="n">
         <v>0</v>
@@ -49269,7 +49253,7 @@
         <v>1983.5</v>
       </c>
       <c r="AV2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AW2" t="n">
         <v>0</v>
@@ -49458,7 +49442,7 @@
         <v>4682</v>
       </c>
       <c r="AV3" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AW3" t="n">
         <v>0</v>
@@ -49938,7 +49922,7 @@
         <v>1734</v>
       </c>
       <c r="AV2" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="AW2" t="n">
         <v>0</v>
@@ -50123,7 +50107,7 @@
         <v>1771</v>
       </c>
       <c r="AV3" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="AW3" t="n">
         <v>0</v>
@@ -50308,7 +50292,7 @@
         <v>4985</v>
       </c>
       <c r="AV4" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="AW4" t="n">
         <v>0</v>
@@ -50493,7 +50477,7 @@
         <v>7158</v>
       </c>
       <c r="AV5" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AW5" t="n">
         <v>0</v>
@@ -50678,7 +50662,7 @@
         <v>5618</v>
       </c>
       <c r="AV6" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="AW6" t="n">
         <v>0</v>
@@ -50867,7 +50851,7 @@
         <v>1833</v>
       </c>
       <c r="AV7" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AW7" t="n">
         <v>0</v>
@@ -51056,7 +51040,7 @@
         <v>173.2</v>
       </c>
       <c r="AV8" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AW8" t="n">
         <v>0</v>
@@ -51241,7 +51225,7 @@
         <v>16435</v>
       </c>
       <c r="AV9" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="AW9" t="n">
         <v>0</v>

</xml_diff>